<commit_message>
Add homework assignments HW9, HW10, HW11, and HW12
- Created HW9.md for chapter 2 of the GitKit book, covering Git settings and repository management.
- Created HW10.md for chapter 3 of the GitKit book, focusing on local operations and upstreaming changes.
- Created HW11.md for chapter 4 of the GitKit book, detailing synchronization with upstream repositories.
- Created HW12.md for chapter 5 of the GitKit book, addressing handling merge conflicts.
</commit_message>
<xml_diff>
--- a/docs/comp190-schedule-8-21-2026.xlsx
+++ b/docs/comp190-schedule-8-21-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jmac\git\comp190-web\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A045674F-F6E1-4300-A2B4-A64353E748E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60455259-5083-454F-A4C6-39AA11815765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Course Schedule" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="58">
   <si>
     <t>Date</t>
   </si>
@@ -122,9 +122,6 @@
     <t>Homework due</t>
   </si>
   <si>
-    <t>Fri</t>
-  </si>
-  <si>
     <t>Operating Systems, Docker and Linux</t>
   </si>
   <si>
@@ -201,9 +198,6 @@
   </si>
   <si>
     <t>AI and Intellectual Property</t>
-  </si>
-  <si>
-    <t>HW14</t>
   </si>
   <si>
     <t>wrapup</t>
@@ -365,7 +359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -390,44 +384,38 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -731,21 +719,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.140625" customWidth="1"/>
-    <col min="2" max="2" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" customWidth="1"/>
-    <col min="6" max="6" width="42.140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.1796875" customWidth="1"/>
+    <col min="2" max="2" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.26953125" customWidth="1"/>
+    <col min="6" max="6" width="42.1796875" style="1" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="13.453125" customWidth="1"/>
     <col min="9" max="9" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="37" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>15</v>
       </c>
@@ -768,10 +756,10 @@
         <v>28</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="42" x14ac:dyDescent="0.45">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -785,19 +773,19 @@
         <f>A2</f>
         <v>1</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>30</v>
+      <c r="F2" s="10" t="s">
+        <v>29</v>
       </c>
       <c r="G2" s="7"/>
       <c r="H2" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A3" s="7">
         <v>2</v>
       </c>
@@ -812,19 +800,19 @@
         <f t="shared" ref="D3:D8" si="0">A3</f>
         <v>2</v>
       </c>
-      <c r="E3" s="16"/>
-      <c r="F3" s="11" t="s">
-        <v>31</v>
+      <c r="E3" s="15"/>
+      <c r="F3" s="10" t="s">
+        <v>30</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>1</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I3" s="3"/>
     </row>
-    <row r="4" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A4" s="7">
         <v>3</v>
       </c>
@@ -839,19 +827,19 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="E4" s="16"/>
-      <c r="F4" s="11" t="s">
-        <v>32</v>
+      <c r="E4" s="15"/>
+      <c r="F4" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="G4" s="7" t="s">
         <v>2</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I4" s="3"/>
     </row>
-    <row r="5" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -866,19 +854,19 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="E5" s="16"/>
-      <c r="F5" s="11" t="s">
-        <v>33</v>
+      <c r="E5" s="15"/>
+      <c r="F5" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="G5" s="7" t="s">
         <v>3</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I5" s="3"/>
     </row>
-    <row r="6" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -893,19 +881,19 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="E6" s="16"/>
-      <c r="F6" s="11" t="s">
-        <v>34</v>
+      <c r="E6" s="15"/>
+      <c r="F6" s="10" t="s">
+        <v>33</v>
       </c>
       <c r="G6" s="7" t="s">
         <v>4</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I6" s="3"/>
     </row>
-    <row r="7" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="42" x14ac:dyDescent="0.45">
       <c r="A7" s="7">
         <v>6</v>
       </c>
@@ -920,21 +908,21 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="E7" s="16" t="s">
+      <c r="E7" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="11" t="s">
-        <v>35</v>
+      <c r="F7" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="G7" s="7" t="s">
         <v>5</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I7" s="3"/>
     </row>
-    <row r="8" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A8" s="7">
         <v>7</v>
       </c>
@@ -949,32 +937,32 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="E8" s="16"/>
-      <c r="F8" s="11" t="s">
-        <v>36</v>
+      <c r="E8" s="15"/>
+      <c r="F8" s="10" t="s">
+        <v>35</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I8" s="3"/>
     </row>
-    <row r="9" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A9" s="14" t="s">
+    <row r="9" spans="1:9" ht="21" x14ac:dyDescent="0.45">
+      <c r="A9" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="11"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="10"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="3"/>
     </row>
-    <row r="10" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A10" s="7">
         <v>8</v>
       </c>
@@ -988,19 +976,19 @@
       <c r="D10" s="9">
         <v>8</v>
       </c>
-      <c r="E10" s="16"/>
-      <c r="F10" s="11" t="s">
-        <v>55</v>
+      <c r="E10" s="15"/>
+      <c r="F10" s="10" t="s">
+        <v>54</v>
       </c>
       <c r="G10" s="7" t="s">
         <v>7</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="7">
         <v>9</v>
       </c>
@@ -1014,21 +1002,21 @@
       <c r="D11" s="9">
         <v>9</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="F11" s="11" t="s">
-        <v>37</v>
+      <c r="F11" s="10" t="s">
+        <v>36</v>
       </c>
       <c r="G11" s="7" t="s">
         <v>8</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I11" s="3"/>
     </row>
-    <row r="12" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A12" s="7">
         <v>10</v>
       </c>
@@ -1042,19 +1030,19 @@
       <c r="D12" s="9">
         <v>10</v>
       </c>
-      <c r="E12" s="18"/>
-      <c r="F12" s="11" t="s">
-        <v>38</v>
+      <c r="E12" s="17"/>
+      <c r="F12" s="10" t="s">
+        <v>37</v>
       </c>
       <c r="G12" s="7" t="s">
         <v>9</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I12" s="3"/>
     </row>
-    <row r="13" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A13" s="7">
         <v>11</v>
       </c>
@@ -1068,19 +1056,19 @@
       <c r="D13" s="9">
         <v>11</v>
       </c>
-      <c r="E13" s="18"/>
-      <c r="F13" s="11" t="s">
-        <v>39</v>
+      <c r="E13" s="17"/>
+      <c r="F13" s="10" t="s">
+        <v>38</v>
       </c>
       <c r="G13" s="7" t="s">
         <v>10</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I13" s="3"/>
     </row>
-    <row r="14" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A14" s="7">
         <v>12</v>
       </c>
@@ -1094,32 +1082,32 @@
       <c r="D14" s="9">
         <v>12</v>
       </c>
-      <c r="E14" s="18"/>
-      <c r="F14" s="11" t="s">
-        <v>40</v>
+      <c r="E14" s="17"/>
+      <c r="F14" s="10" t="s">
+        <v>39</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>11</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I14" s="3"/>
     </row>
-    <row r="15" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
+    <row r="15" spans="1:9" ht="21" x14ac:dyDescent="0.45">
+      <c r="A15" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="11"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="10"/>
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" s="3"/>
     </row>
-    <row r="16" spans="1:9" ht="40.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="42" x14ac:dyDescent="0.45">
       <c r="A16" s="7">
         <v>13</v>
       </c>
@@ -1133,21 +1121,21 @@
       <c r="D16" s="9">
         <v>13</v>
       </c>
-      <c r="E16" s="16" t="s">
+      <c r="E16" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>58</v>
+      <c r="F16" s="10" t="s">
+        <v>56</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>12</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" ht="21" x14ac:dyDescent="0.45">
       <c r="A17" s="7">
         <v>14</v>
       </c>
@@ -1161,54 +1149,37 @@
       <c r="D17" s="9">
         <v>14</v>
       </c>
-      <c r="E17" s="16"/>
-      <c r="F17" s="12" t="s">
-        <v>57</v>
+      <c r="E17" s="15"/>
+      <c r="F17" s="10" t="s">
+        <v>55</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" s="8">
-        <f>C17+2</f>
-        <v>46367</v>
-      </c>
-      <c r="D18" s="9"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:9" s="22" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20" t="s">
+    <row r="18" spans="1:9" s="13" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="11"/>
+      <c r="B18" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C19" s="21">
+      <c r="C18" s="12">
         <v>46375</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D18" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D18:F18"/>
     <mergeCell ref="E7:E10"/>
     <mergeCell ref="E16:E17"/>
     <mergeCell ref="E11:E15"/>

</xml_diff>